<commit_message>
strategy & 2026 data
</commit_message>
<xml_diff>
--- a/data/source/driver_default.xlsx
+++ b/data/source/driver_default.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76929c7f1b9de68b/Documents/Dada/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="11_EDD44E5993BC482A58B3BF0BF84E774AB1880010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98967749-825B-4DC3-B1F2-6CAE14CF24E8}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="11_EDD44E5993BC482A58B3BF0BF84E774AB1880010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EED6528-C961-45D1-91A4-58843A4B1AC9}"/>
   <bookViews>
     <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>name</t>
   </si>
@@ -116,12 +116,6 @@
     <t>ALO</t>
   </si>
   <si>
-    <t>Yuki Tsunoda</t>
-  </si>
-  <si>
-    <t>TSU</t>
-  </si>
-  <si>
     <t>Alexander Albon</t>
   </si>
   <si>
@@ -165,6 +159,24 @@
   </si>
   <si>
     <t>BOR</t>
+  </si>
+  <si>
+    <t>Arvid Lindblad</t>
+  </si>
+  <si>
+    <t>LIN</t>
+  </si>
+  <si>
+    <t>Valterri Bottas</t>
+  </si>
+  <si>
+    <t>BOT</t>
+  </si>
+  <si>
+    <t>Sergio Pérez</t>
+  </si>
+  <si>
+    <t>PER</t>
   </si>
 </sst>
 </file>
@@ -220,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -232,6 +244,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -249,10 +264,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -543,15 +554,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -562,127 +574,127 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D6">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D7">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D8">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C9" s="3">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D9">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C10" s="3">
         <v>89</v>
@@ -691,12 +703,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="C11" s="3">
         <v>89</v>
@@ -705,82 +717,82 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C12" s="3">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D12">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C13" s="3">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D13">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D14">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C15" s="3">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D15">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D16">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C17" s="3">
         <v>89</v>
@@ -789,65 +801,93 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C18" s="3">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D18">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="C19" s="3">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D19">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C20" s="3">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C21" s="3">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D21">
         <v>10</v>
       </c>
     </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="5">
+        <v>86</v>
+      </c>
+      <c r="D22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="5">
+        <v>86</v>
+      </c>
+      <c r="D23">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D21">
-    <sortCondition ref="D3:D21"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D23">
+    <sortCondition ref="D8:D23"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
big update, big correction
</commit_message>
<xml_diff>
--- a/data/source/driver_default.xlsx
+++ b/data/source/driver_default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76929c7f1b9de68b/Documents/Dada/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="11_EDD44E5993BC482A58B3BF0BF84E774AB1880010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EED6528-C961-45D1-91A4-58843A4B1AC9}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="11_EDD44E5993BC482A58B3BF0BF84E774AB1880010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F89585BF-AD21-401E-8E5F-FC39FBF0DC14}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -232,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -244,9 +244,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -613,7 +610,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="3">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -627,7 +624,7 @@
         <v>31</v>
       </c>
       <c r="C5" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -683,7 +680,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="3">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -781,7 +778,7 @@
         <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16">
         <v>8</v>
@@ -823,7 +820,7 @@
         <v>41</v>
       </c>
       <c r="C19" s="3">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D19">
         <v>9</v>
@@ -864,7 +861,7 @@
       <c r="B22" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="4">
         <v>86</v>
       </c>
       <c r="D22">
@@ -878,7 +875,7 @@
       <c r="B23" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="4">
         <v>86</v>
       </c>
       <c r="D23">

</xml_diff>

<commit_message>
scoring, gp, fin et dnf stats takes sprint races into account
</commit_message>
<xml_diff>
--- a/data/source/driver_default.xlsx
+++ b/data/source/driver_default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76929c7f1b9de68b/Documents/Dada/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="155" documentId="11_EDD44E5993BC482A58B3BF0BF84E774AB1880010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F89585BF-AD21-401E-8E5F-FC39FBF0DC14}"/>
+  <xr:revisionPtr revIDLastSave="179" documentId="11_EDD44E5993BC482A58B3BF0BF84E774AB1880010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B80AF70E-A6B3-4B67-845B-D9D5B0AA5438}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
   <si>
     <t>name</t>
   </si>
@@ -177,6 +177,54 @@
   </si>
   <si>
     <t>PER</t>
+  </si>
+  <si>
+    <t>flag</t>
+  </si>
+  <si>
+    <t>uk.png</t>
+  </si>
+  <si>
+    <t>australia.png</t>
+  </si>
+  <si>
+    <t>italy.png</t>
+  </si>
+  <si>
+    <t>netherlands.png</t>
+  </si>
+  <si>
+    <t>france.png</t>
+  </si>
+  <si>
+    <t>monaco.png</t>
+  </si>
+  <si>
+    <t>thailand.png</t>
+  </si>
+  <si>
+    <t>spain.png</t>
+  </si>
+  <si>
+    <t>new_zealand.png</t>
+  </si>
+  <si>
+    <t>canada.png</t>
+  </si>
+  <si>
+    <t>germany.png</t>
+  </si>
+  <si>
+    <t>brazil.png</t>
+  </si>
+  <si>
+    <t>argentina.png</t>
+  </si>
+  <si>
+    <t>finland.png</t>
+  </si>
+  <si>
+    <t>mexico.png</t>
   </si>
 </sst>
 </file>
@@ -232,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -245,6 +293,9 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -261,6 +312,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -551,16 +606,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -573,8 +629,11 @@
       <c r="D1" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -587,8 +646,11 @@
       <c r="D2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -601,8 +663,11 @@
       <c r="D3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -615,8 +680,11 @@
       <c r="D4">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -629,8 +697,11 @@
       <c r="D5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -643,8 +714,11 @@
       <c r="D6">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -657,8 +731,11 @@
       <c r="D7">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -671,8 +748,11 @@
       <c r="D8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -685,8 +765,11 @@
       <c r="D9">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -699,8 +782,11 @@
       <c r="D10">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -713,8 +799,11 @@
       <c r="D11">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -727,8 +816,11 @@
       <c r="D12">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -741,8 +833,11 @@
       <c r="D13">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -755,8 +850,11 @@
       <c r="D14">
         <v>7</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -769,8 +867,11 @@
       <c r="D15">
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -783,8 +884,11 @@
       <c r="D16">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -797,8 +901,11 @@
       <c r="D17">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -811,8 +918,11 @@
       <c r="D18">
         <v>9</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -825,8 +935,11 @@
       <c r="D19">
         <v>9</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -839,8 +952,11 @@
       <c r="D20">
         <v>10</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -853,8 +969,11 @@
       <c r="D21">
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -867,8 +986,11 @@
       <c r="D22">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>46</v>
       </c>
@@ -880,6 +1002,9 @@
       </c>
       <c r="D23">
         <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>